<commit_message>
chore(samples): give the second coverage form minimum times and correct its platform notes
Speed violations and comments work in web forms; only audio audits need
SurveyCTO Collect. resp_name and hh_size get a minimum time so that speed
violations can be recorded.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/coverage2/ctosim_coverage2.xlsx
+++ b/samples/coverage2/ctosim_coverage2.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K37"/>
+  <dimension ref="A1:L37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -474,6 +474,11 @@
           <t>repeat_count</t>
         </is>
       </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>minimum_seconds</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -716,12 +721,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Respondent's first name (fictitious)</t>
+          <t>Respondent's first name (fictitious; answer in under 10 seconds)</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
           <t>yes</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>10</t>
         </is>
       </c>
     </row>
@@ -782,7 +792,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Number of household members (1 to 3 for this test)</t>
+          <t>Number of household members (1 to 3 for this test; answer in under 10 seconds)</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -793,6 +803,11 @@
       <c r="I19" t="inlineStr">
         <is>
           <t>yes</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>10</t>
         </is>
       </c>
     </row>

</xml_diff>